<commit_message>
Add ANSI colored console outputs (Yellow=Neutral, Green=Buy, Red=Sell), instant Excel sync on close, and full M15 trade history sync
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -6711,7 +6711,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>&gt;= 58.0% + Dynamic AI Exit ($1.50 TP / AI Cut-Loss)</t>
+          <t>&gt;= 58.0% + Dynamic AI Exit (.50 TP / AI Cut-Loss)</t>
         </is>
       </c>
     </row>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-09 13:50:00 WIB</t>
+          <t>2026-09-09 17:55:32 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add live probability percentage display on console line, startup market audit, and silent background Excel sync
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -6711,7 +6711,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>&gt;= 58.0% + Dynamic AI Exit (.50 TP / AI Cut-Loss)</t>
+          <t>&gt;= 58.0% + Dynamic AI Exit ($1.50 TP / AI Cut-Loss)</t>
         </is>
       </c>
     </row>
@@ -6831,7 +6831,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-09 17:55:32 WIB</t>
+          <t>2026-09-09 18:06:50 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement SMC Key-Level Bounce Scalper for M5, Single Instance Lock, and Unified Desktop GUI Dashboard with Tabbed Controls
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q89"/>
+  <dimension ref="A1:Q100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1893,11 +1893,11 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>2513410135</v>
+        <v>2513356937</v>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08 21:55:00</t>
+          <t>2026-09-08 21:50:00</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>4m 48d</t>
+          <t>9m 48d</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1924,22 +1924,22 @@
         <v>0.01</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>4392.736</v>
+        <v>4393.196</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>4398.021</v>
+        <v>4398.168</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>4386.721</v>
+        <v>4386.868</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>4398.021</v>
+        <v>4398.168</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>-52.8</v>
+        <v>-49.7</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>-5.28</v>
+        <v>-4.97</v>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
@@ -1962,11 +1962,11 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>2513356937</v>
+        <v>2513410135</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08 21:50:00</t>
+          <t>2026-09-08 21:55:00</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>9m 48d</t>
+          <t>4m 48d</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1993,22 +1993,22 @@
         <v>0.01</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>4393.196</v>
+        <v>4392.736</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>4398.168</v>
+        <v>4398.021</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>4386.868</v>
+        <v>4386.721</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>4398.168</v>
+        <v>4398.021</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>-49.7</v>
+        <v>-52.8</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>-4.97</v>
+        <v>-5.28</v>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
@@ -3204,11 +3204,11 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="n">
-        <v>2514126126</v>
+        <v>2514152997</v>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08 23:55:00</t>
+          <t>2026-09-08 23:59:59</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>7m 17d</t>
+          <t>2m 18d</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -3235,22 +3235,22 @@
         <v>0.01</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>4394.151</v>
+        <v>4393.793</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>4397.495</v>
+        <v>4397.493</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>4388.195</v>
+        <v>4388.193</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>4397.893</v>
+        <v>4397.988</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>-37.4</v>
+        <v>-42</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>-3.74</v>
+        <v>-4.2</v>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
@@ -3273,11 +3273,11 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="n">
-        <v>2514152997</v>
+        <v>2514126126</v>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08 23:59:59</t>
+          <t>2026-09-08 23:55:00</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>2m 18d</t>
+          <t>7m 17d</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -3304,22 +3304,22 @@
         <v>0.01</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>4393.793</v>
+        <v>4394.151</v>
       </c>
       <c r="J41" s="4" t="n">
-        <v>4397.493</v>
+        <v>4397.495</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>4388.193</v>
+        <v>4388.195</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>4397.988</v>
+        <v>4397.893</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>-42</v>
+        <v>-37.4</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>-4.2</v>
+        <v>-3.74</v>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
@@ -4101,11 +4101,11 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="n">
-        <v>2515114548</v>
+        <v>2515148608</v>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09 05:39:52</t>
+          <t>2026-09-09 06:05:00</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -4115,7 +4115,7 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>46m 54d</t>
+          <t>21m 46d</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -4132,22 +4132,22 @@
         <v>0.01</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>4352.809</v>
+        <v>4353.34</v>
       </c>
       <c r="J53" s="4" t="n">
-        <v>4355.709</v>
+        <v>4355.84</v>
       </c>
       <c r="K53" s="4" t="n">
-        <v>4348.409</v>
+        <v>4349.54</v>
       </c>
       <c r="L53" s="3" t="n">
-        <v>4355.709</v>
+        <v>4355.84</v>
       </c>
       <c r="M53" s="4" t="n">
-        <v>-29</v>
+        <v>-25</v>
       </c>
       <c r="N53" s="3" t="n">
-        <v>-2.9</v>
+        <v>-2.5</v>
       </c>
       <c r="O53" s="4" t="inlineStr">
         <is>
@@ -4170,11 +4170,11 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="n">
-        <v>2515148608</v>
+        <v>2515114548</v>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09 06:05:00</t>
+          <t>2026-09-09 05:39:52</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>21m 46d</t>
+          <t>46m 54d</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -4201,22 +4201,22 @@
         <v>0.01</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>4353.34</v>
+        <v>4352.809</v>
       </c>
       <c r="J54" s="4" t="n">
-        <v>4355.84</v>
+        <v>4355.709</v>
       </c>
       <c r="K54" s="4" t="n">
-        <v>4349.54</v>
+        <v>4348.409</v>
       </c>
       <c r="L54" s="3" t="n">
-        <v>4355.84</v>
+        <v>4355.709</v>
       </c>
       <c r="M54" s="4" t="n">
-        <v>-25</v>
+        <v>-29</v>
       </c>
       <c r="N54" s="3" t="n">
-        <v>-2.5</v>
+        <v>-2.9</v>
       </c>
       <c r="O54" s="4" t="inlineStr">
         <is>
@@ -4239,11 +4239,11 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="n">
-        <v>2515223561</v>
+        <v>2515208352</v>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09 06:45:00</t>
+          <t>2026-09-09 06:35:00</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>4m 22d</t>
+          <t>14m 22d</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -4270,22 +4270,22 @@
         <v>0.01</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>4358.359</v>
+        <v>4358.87</v>
       </c>
       <c r="J55" s="4" t="n">
-        <v>4361.142</v>
+        <v>4361.37</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>4354.842</v>
+        <v>4355.07</v>
       </c>
       <c r="L55" s="3" t="n">
-        <v>4354.842</v>
+        <v>4355.07</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>35.2</v>
+        <v>38</v>
       </c>
       <c r="N55" s="3" t="n">
-        <v>3.52</v>
+        <v>3.8</v>
       </c>
       <c r="O55" s="4" t="inlineStr">
         <is>
@@ -4308,11 +4308,11 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="n">
-        <v>2515208352</v>
+        <v>2515223561</v>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09 06:35:00</t>
+          <t>2026-09-09 06:45:00</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>14m 22d</t>
+          <t>4m 22d</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -4339,22 +4339,22 @@
         <v>0.01</v>
       </c>
       <c r="I56" s="4" t="n">
-        <v>4358.87</v>
+        <v>4358.359</v>
       </c>
       <c r="J56" s="4" t="n">
-        <v>4361.37</v>
+        <v>4361.142</v>
       </c>
       <c r="K56" s="4" t="n">
-        <v>4355.07</v>
+        <v>4354.842</v>
       </c>
       <c r="L56" s="3" t="n">
-        <v>4355.07</v>
+        <v>4354.842</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>38</v>
+        <v>35.2</v>
       </c>
       <c r="N56" s="3" t="n">
-        <v>3.8</v>
+        <v>3.52</v>
       </c>
       <c r="O56" s="4" t="inlineStr">
         <is>
@@ -4791,11 +4791,11 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="n">
-        <v>2515795700</v>
+        <v>2515759279</v>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09 08:44:59</t>
+          <t>2026-09-09 08:34:59</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>48m 10d</t>
+          <t>58m 10d</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -4822,22 +4822,22 @@
         <v>0.01</v>
       </c>
       <c r="I63" s="4" t="n">
-        <v>4376.398</v>
+        <v>4376.694</v>
       </c>
       <c r="J63" s="4" t="n">
-        <v>4380.712</v>
+        <v>4381.094</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>4370.012</v>
+        <v>4370.094</v>
       </c>
       <c r="L63" s="3" t="n">
-        <v>4370.012</v>
+        <v>4370.094</v>
       </c>
       <c r="M63" s="4" t="n">
-        <v>63.9</v>
+        <v>66</v>
       </c>
       <c r="N63" s="3" t="n">
-        <v>6.39</v>
+        <v>6.6</v>
       </c>
       <c r="O63" s="4" t="inlineStr">
         <is>
@@ -4860,11 +4860,11 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="n">
-        <v>2515759279</v>
+        <v>2515795700</v>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09 08:34:59</t>
+          <t>2026-09-09 08:44:59</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>58m 10d</t>
+          <t>48m 10d</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -4891,22 +4891,22 @@
         <v>0.01</v>
       </c>
       <c r="I64" s="4" t="n">
-        <v>4376.694</v>
+        <v>4376.398</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>4381.094</v>
+        <v>4380.712</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>4370.094</v>
+        <v>4370.012</v>
       </c>
       <c r="L64" s="3" t="n">
-        <v>4370.094</v>
+        <v>4370.012</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>66</v>
+        <v>63.9</v>
       </c>
       <c r="N64" s="3" t="n">
-        <v>6.6</v>
+        <v>6.39</v>
       </c>
       <c r="O64" s="4" t="inlineStr">
         <is>
@@ -6644,6 +6644,765 @@
         </is>
       </c>
       <c r="Q89" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="3" t="n">
+        <v>2518262642</v>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 18:09:55</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 18:45:48</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>35m 53d</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I90" s="4" t="n">
+        <v>4404.564</v>
+      </c>
+      <c r="J90" s="4" t="n">
+        <v>4400.564</v>
+      </c>
+      <c r="K90" s="4" t="n">
+        <v>4419.564</v>
+      </c>
+      <c r="L90" s="3" t="n">
+        <v>4406.115</v>
+      </c>
+      <c r="M90" s="4" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="N90" s="3" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="O90" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P90" s="4" t="inlineStr">
+        <is>
+          <t>Bot Dynamic Scalp TP</t>
+        </is>
+      </c>
+      <c r="Q90" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="n">
+        <v>2518428443</v>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 18:44:55</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 18:49:02</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>4m 7d</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I91" s="4" t="n">
+        <v>4405.636</v>
+      </c>
+      <c r="J91" s="4" t="n">
+        <v>4401.636</v>
+      </c>
+      <c r="K91" s="4" t="n">
+        <v>4420.636</v>
+      </c>
+      <c r="L91" s="3" t="n">
+        <v>4408.392</v>
+      </c>
+      <c r="M91" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="N91" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="O91" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P91" s="4" t="inlineStr">
+        <is>
+          <t>Bot Dynamic Scalp TP</t>
+        </is>
+      </c>
+      <c r="Q91" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="3" t="n">
+        <v>2519397460</v>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 20:39:55</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 20:42:02</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>2m 7d</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I92" s="4" t="n">
+        <v>4421.782</v>
+      </c>
+      <c r="J92" s="4" t="n">
+        <v>4417.782</v>
+      </c>
+      <c r="K92" s="4" t="n">
+        <v>4436.782</v>
+      </c>
+      <c r="L92" s="3" t="n">
+        <v>4417.782</v>
+      </c>
+      <c r="M92" s="4" t="n">
+        <v>-40</v>
+      </c>
+      <c r="N92" s="3" t="n">
+        <v>-4</v>
+      </c>
+      <c r="O92" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P92" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q92" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="3" t="n">
+        <v>2519575193</v>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 20:54:55</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 20:55:22</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>0m 27d</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I93" s="4" t="n">
+        <v>4415.842</v>
+      </c>
+      <c r="J93" s="4" t="n">
+        <v>4411.842</v>
+      </c>
+      <c r="K93" s="4" t="n">
+        <v>4430.842</v>
+      </c>
+      <c r="L93" s="3" t="n">
+        <v>4416.311</v>
+      </c>
+      <c r="M93" s="4" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="N93" s="3" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="O93" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P93" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q93" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="3" t="n">
+        <v>2519685035</v>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 21:04:55</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 21:05:05</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>0m 10d</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I94" s="4" t="n">
+        <v>4422.948</v>
+      </c>
+      <c r="J94" s="4" t="n">
+        <v>4418.948</v>
+      </c>
+      <c r="K94" s="4" t="n">
+        <v>4437.948</v>
+      </c>
+      <c r="L94" s="3" t="n">
+        <v>4424.881</v>
+      </c>
+      <c r="M94" s="4" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="N94" s="3" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="O94" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P94" s="4" t="inlineStr">
+        <is>
+          <t>Bot Dynamic Scalp TP</t>
+        </is>
+      </c>
+      <c r="Q94" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="3" t="n">
+        <v>2520080463</v>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 21:49:55</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 21:50:59</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>1m 4d</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I95" s="4" t="n">
+        <v>4421.454</v>
+      </c>
+      <c r="J95" s="4" t="n">
+        <v>4417.454</v>
+      </c>
+      <c r="K95" s="4" t="n">
+        <v>4436.454</v>
+      </c>
+      <c r="L95" s="3" t="n">
+        <v>4421.961</v>
+      </c>
+      <c r="M95" s="4" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="N95" s="3" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="O95" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P95" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q95" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="3" t="n">
+        <v>2520808066</v>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 22:39:55</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 22:40:03</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>0m 8d</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I96" s="4" t="n">
+        <v>4403.160000000001</v>
+      </c>
+      <c r="J96" s="4" t="n">
+        <v>4399.214</v>
+      </c>
+      <c r="K96" s="4" t="n">
+        <v>4418.214</v>
+      </c>
+      <c r="L96" s="3" t="n">
+        <v>4405.962</v>
+      </c>
+      <c r="M96" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="N96" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O96" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P96" s="4" t="inlineStr">
+        <is>
+          <t>Bot Dynamic Scalp TP</t>
+        </is>
+      </c>
+      <c r="Q96" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="3" t="n">
+        <v>2520808306</v>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 22:39:55</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 22:40:22</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>0m 27d</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I97" s="4" t="n">
+        <v>4404.783</v>
+      </c>
+      <c r="J97" s="4" t="n">
+        <v>4400.823</v>
+      </c>
+      <c r="K97" s="4" t="n">
+        <v>4419.823</v>
+      </c>
+      <c r="L97" s="3" t="n">
+        <v>4400.823</v>
+      </c>
+      <c r="M97" s="4" t="n">
+        <v>-39.6</v>
+      </c>
+      <c r="N97" s="3" t="n">
+        <v>-3.96</v>
+      </c>
+      <c r="O97" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P97" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q97" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="3" t="n">
+        <v>2520907026</v>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 22:54:56</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:00:11</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>5m 15d</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I98" s="4" t="n">
+        <v>4401.351</v>
+      </c>
+      <c r="J98" s="4" t="n">
+        <v>4397.212</v>
+      </c>
+      <c r="K98" s="4" t="n">
+        <v>4416.212</v>
+      </c>
+      <c r="L98" s="3" t="n">
+        <v>4397.212</v>
+      </c>
+      <c r="M98" s="4" t="n">
+        <v>-41.4</v>
+      </c>
+      <c r="N98" s="3" t="n">
+        <v>-4.14</v>
+      </c>
+      <c r="O98" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P98" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q98" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="3" t="n">
+        <v>2520962727</v>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:04:56</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09 23:06:09</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>1m 13d</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I99" s="4" t="n">
+        <v>4402.761</v>
+      </c>
+      <c r="J99" s="4" t="n">
+        <v>4398.759</v>
+      </c>
+      <c r="K99" s="4" t="n">
+        <v>4417.759</v>
+      </c>
+      <c r="L99" s="3" t="n">
+        <v>4398.759</v>
+      </c>
+      <c r="M99" s="4" t="n">
+        <v>-40</v>
+      </c>
+      <c r="N99" s="3" t="n">
+        <v>-4</v>
+      </c>
+      <c r="O99" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P99" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q99" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 Dynamic Scalper</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="3" t="n">
+        <v>2521682888</v>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:49:56</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10 01:56:32</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>6m 36d</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I100" s="4" t="n">
+        <v>4407.119</v>
+      </c>
+      <c r="J100" s="4" t="n">
+        <v>4403.139</v>
+      </c>
+      <c r="K100" s="4" t="n">
+        <v>4422.139</v>
+      </c>
+      <c r="L100" s="3" t="n">
+        <v>4403.139</v>
+      </c>
+      <c r="M100" s="4" t="n">
+        <v>-39.8</v>
+      </c>
+      <c r="N100" s="3" t="n">
+        <v>-3.98</v>
+      </c>
+      <c r="O100" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P100" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q100" s="4" t="inlineStr">
         <is>
           <t>LightGBM M5 Dynamic Scalper</t>
         </is>
@@ -6735,7 +7494,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>88 Trade</t>
+          <t>99 Trade</t>
         </is>
       </c>
     </row>
@@ -6747,7 +7506,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>88.0%</t>
+          <t>99.0%</t>
         </is>
       </c>
     </row>
@@ -6759,7 +7518,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>37 Trade</t>
+          <t>43 Trade</t>
         </is>
       </c>
     </row>
@@ -6771,7 +7530,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>51 Trade</t>
+          <t>56 Trade</t>
         </is>
       </c>
     </row>
@@ -6783,7 +7542,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>42.05%</t>
+          <t>43.43%</t>
         </is>
       </c>
     </row>
@@ -6795,7 +7554,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>$+28.72 USD</t>
+          <t>$+18.66 USD</t>
         </is>
       </c>
     </row>
@@ -6807,7 +7566,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>$+0.33 USD</t>
+          <t>$+0.19 USD</t>
         </is>
       </c>
     </row>
@@ -6819,7 +7578,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.09</t>
         </is>
       </c>
     </row>
@@ -6831,7 +7590,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-09 18:43:02 WIB</t>
+          <t>2026-09-10 01:58:20 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix UTF-8 subprocess pipe decoding in GUI, differentiate manual stop from process exit, and improve live countdown rendering
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -7470,7 +7470,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>&gt;= 58.0% + Dynamic AI Exit ($1.50 TP / AI Cut-Loss)</t>
+          <t>SMC Level Bounce (TP $2.00 / Cut-Loss $1.80)</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10 01:58:20 WIB</t>
+          <t>2026-09-10 02:09:36 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement Macro_Economic_News_Engine (CPI, PPI, NFP, FOMC), Dynamic ATR Breathing Room (anti-kejilat SL), and Trend-Aware Momentum logic v3.5
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
@@ -1883,6 +1883,696 @@
         </is>
       </c>
       <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>2533562125</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:29:54</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:56:41</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>26m 47d</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>4349.17</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>4352.37</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>4339.17</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>4339.17</v>
+      </c>
+      <c r="M21" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>Hit Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>2533679472</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 17:59:55</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:00:46</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>0m 51d</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>4337.891000000001</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>4341.091</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>4327.891</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>4340.335</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>-2.45</v>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>AI Early Cut-Loss (Reversal)</t>
+        </is>
+      </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>2533728294</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:09:54</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:22:04</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>12m 10d</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>4337.442</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>4340.642</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>4327.442</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>4339.914</v>
+      </c>
+      <c r="M23" s="4" t="n">
+        <v>-24.7</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>-2.47</v>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t>AI Early Cut-Loss (Reversal)</t>
+        </is>
+      </c>
+      <c r="Q23" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>2533850578</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:34:54</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:45:00</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>10m 6d</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>4332.001</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>4335.201</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>4322.001</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>4334.862</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>-28.6</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>AI Early Cut-Loss (Reversal)</t>
+        </is>
+      </c>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>2533940785</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:54:54</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:59:13</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>4m 19d</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>4331.819</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>4335.019</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>4321.819</v>
+      </c>
+      <c r="L25" s="3" t="n">
+        <v>4334.239</v>
+      </c>
+      <c r="M25" s="4" t="n">
+        <v>-24.2</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>-2.42</v>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="inlineStr">
+        <is>
+          <t>AI Early Cut-Loss (Reversal)</t>
+        </is>
+      </c>
+      <c r="Q25" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>2533960848</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:59:54</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 19:27:33</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>27m 39d</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>4332.929</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>4336.349</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>4323.149</v>
+      </c>
+      <c r="L26" s="3" t="n">
+        <v>4336.349</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>-34.2</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>-3.42</v>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2534427120</v>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 19:34:54</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 19:36:01</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>1m 7d</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>4333.126</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>4336.326</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>4323.126</v>
+      </c>
+      <c r="L27" s="3" t="n">
+        <v>4336.326</v>
+      </c>
+      <c r="M27" s="4" t="n">
+        <v>-32</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>-3.2</v>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P27" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q27" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>2534781964</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 19:49:54</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 19:50:20</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>0m 26d</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>4363.148</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>4366.348</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>4353.148</v>
+      </c>
+      <c r="L28" s="3" t="n">
+        <v>4362.916</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P28" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q28" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>2535133628</v>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:09:54</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:11:26</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>1m 32d</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>4384.329</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>4387.464</v>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>4374.264</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>4383.41</v>
+      </c>
+      <c r="M29" s="4" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.4 (Confluence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>2535493174</v>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:39:54</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:40:00</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>0m 6d</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>4386.908</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>4390.108</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>4376.908</v>
+      </c>
+      <c r="L30" s="3" t="n">
+        <v>4390.61</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>-37</v>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr">
         <is>
           <t>LightGBM M5 v3.4 (Confluence)</t>
         </is>
@@ -1974,7 +2664,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>19 Trade</t>
+          <t>29 Trade</t>
         </is>
       </c>
     </row>
@@ -1986,7 +2676,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>19.0%</t>
+          <t>29.0%</t>
         </is>
       </c>
     </row>
@@ -1998,7 +2688,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>13 Trade</t>
+          <t>16 Trade</t>
         </is>
       </c>
     </row>
@@ -2010,7 +2700,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>6 Trade</t>
+          <t>13 Trade</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2712,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>68.42%</t>
+          <t>55.17%</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2724,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>$+40.40 USD</t>
+          <t>$+31.03 USD</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2736,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>$+2.13 USD</t>
+          <t>$+1.07 USD</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2748,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>1.83</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2760,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-11 17:08:47 WIB</t>
+          <t>2026-09-11 21:16:34 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(execution): resolve NameError latest_atr in execute_auto_trade and harden MT5 order_send
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -487,7 +487,7 @@
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="31" customWidth="1" min="16" max="16"/>
-    <col width="32" customWidth="1" min="17" max="17"/>
+    <col width="33" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -642,7 +642,7 @@
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="Q3" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="Q4" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="Q6" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="Q10" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="Q12" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="Q15" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="Q16" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="Q19" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="Q20" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="Q21" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2022,7 @@
       </c>
       <c r="Q22" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="Q23" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="Q24" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="Q25" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="Q26" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="Q30" s="4" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="64" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.4 (Confluence) (28 Fitur SMC/ICT + DXY + MTF)</t>
+          <t>LightGBM M5 v3.5 (Macro + ATR) (28 Fitur SMC/ICT + DXY + MTF)</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Technical Confluence (Stoch RSI + Patterns v3.4)</t>
+          <t>Macro Calendar Guard + Dynamic ATR v3.5</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-11 21:16:34 WIB</t>
+          <t>2026-09-14 13:55:38 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement v3.7 sniper direct entry, ml retraining dataset logger, and update gui dashboard
- Add Sniper Direct Entry (>=70% probability) in M15 and M5 execution bots to bypass manual heuristic filter lag

- Record full 36 features snapshot at entry into dataset_skenario_ml_retrain.csv for future model fine-tuning

- Update Trading_Bot_GUI_App.py interface title, headers, and parameter cards to v3.7 Sniper

- Reset forward testing logs starting balance to 500 USD with fresh cutoff date (18 Sept 2026 21:55 WIB)

- Add Layer 1 and Layer 2 research evaluation scripts (Pure Model Accuracy & Ideal Execution backtest)

- Add Web Dashboard Server, Cloudflare Tunnel, and organize research documents into ARTIKEL and PRA TA folders
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -7,8 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v3.7)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.7)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v3.6)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.6)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip v3.5)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.5)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip 16-17 Sep)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (Arsip 16-1" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,7 +47,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +58,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -102,6 +120,26 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -468,7 +506,1207 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Trade Ke-</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Ticket Posisi</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Open</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Close</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Durasi</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Simbol</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Tipe</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Entry</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Exit</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Pips (P/L)</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>Saldo ($ USD)</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>Hasil</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t>Keterangan / Alasan Exit</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Model AI</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="84" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Metrik Evaluasi Forward Testing</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Nilai Evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Nama Model</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat) (28 Fitur SMC/ICT + DXY + MTF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Metode Eksekusi</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Otomatis 0-Delay (MetaTrader 5 API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ambang Batas Keyakinan (Threshold)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Versi 3.7 Multi-Zone Scalper (Wide SL + Sniper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Target Forward Testing Skripsi</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>100 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Awal Evaluasi</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>$500.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Terkini</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$500.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Total Trade Otomatis Selesai</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>0 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Progres Evaluasi (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade WIN (Profit)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>0 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade LOSS (Rugi)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>0 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Win Rate (%)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Total Akumulasi Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>$+0.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Return on Investment (ROI)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>+0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Rata-rata Profit per Trade</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>$+0.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Waktu Pembaruan Terakhir</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-19 00:14:55 WIB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="53" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Trade Ke-</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Ticket Posisi</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Open</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Close</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Durasi</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Simbol</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Tipe</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Entry</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Exit</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Pips (P/L)</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>Saldo ($ USD)</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>Hasil</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t>Keterangan / Alasan Exit</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Model AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>2546617136</v>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-15 01:24:54</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-15 02:22:11</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>57m 17d</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I2" s="11" t="n">
+        <v>4308.471</v>
+      </c>
+      <c r="J2" s="11" t="n">
+        <v>4313.971</v>
+      </c>
+      <c r="K2" s="11" t="n">
+        <v>4300.371</v>
+      </c>
+      <c r="L2" s="11" t="n">
+        <v>4300.371</v>
+      </c>
+      <c r="M2" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="N2" s="11" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="O2" s="9" t="n">
+        <v>508.1</v>
+      </c>
+      <c r="P2" s="9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q2" s="10" t="inlineStr">
+        <is>
+          <t>Hit Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="R2" s="10" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>2546768386</v>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-15 02:19:54</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-15 02:34:52</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>14m 58d</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>4301.517</v>
+      </c>
+      <c r="J3" s="11" t="n">
+        <v>4307.017</v>
+      </c>
+      <c r="K3" s="11" t="n">
+        <v>4293.417</v>
+      </c>
+      <c r="L3" s="11" t="n">
+        <v>4293.417</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="N3" s="11" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="O3" s="9" t="n">
+        <v>516.2</v>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q3" s="10" t="inlineStr">
+        <is>
+          <t>Hit Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>2546831919</v>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-15 02:39:54</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-15 02:56:51</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>16m 57d</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>4292.178</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>4297.702</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <v>4284.102</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>4284.102</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="N4" s="11" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="O4" s="9" t="n">
+        <v>524.28</v>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>Hit Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>2549286684</v>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15 14:39:54</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15 14:51:32</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>11m 38d</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>4286.25</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>4280.41</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>4294.96</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>4280.41</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-58.4</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>-5.84</v>
+      </c>
+      <c r="O5" s="12" t="n">
+        <v>518.4400000000001</v>
+      </c>
+      <c r="P5" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R5" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>2549567898</v>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15 15:09:54</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15 15:17:01</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>7m 7d</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>4264.495</v>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>4271.495</v>
+      </c>
+      <c r="K6" s="14" t="n">
+        <v>4251.895</v>
+      </c>
+      <c r="L6" s="14" t="n">
+        <v>4271.495</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N6" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O6" s="12" t="n">
+        <v>511.44</v>
+      </c>
+      <c r="P6" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q6" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R6" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>2550279289</v>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:19:54</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:50:25</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>30m 31d</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>4271.667</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>4278.067</v>
+      </c>
+      <c r="K7" s="14" t="n">
+        <v>4261.947</v>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>4278.067</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <v>-64</v>
+      </c>
+      <c r="N7" s="14" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="O7" s="12" t="n">
+        <v>505.04</v>
+      </c>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R7" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>2550255640</v>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:14:54</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:51:14</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>36m 20d</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>4272.953</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>4279.313</v>
+      </c>
+      <c r="K8" s="14" t="n">
+        <v>4263.303</v>
+      </c>
+      <c r="L8" s="14" t="n">
+        <v>4279.313</v>
+      </c>
+      <c r="M8" s="12" t="n">
+        <v>-63.6</v>
+      </c>
+      <c r="N8" s="14" t="n">
+        <v>-6.36</v>
+      </c>
+      <c r="O8" s="12" t="n">
+        <v>498.68</v>
+      </c>
+      <c r="P8" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R8" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="84" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Metrik Evaluasi Forward Testing</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Nilai Evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Nama Model</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat) (28 Fitur SMC/ICT + DXY + MTF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Metode Eksekusi</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Otomatis 0-Delay (MetaTrader 5 API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ambang Batas Keyakinan (Threshold)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Versi 3.7 Multi-Zone Scalper (Wide SL + Sniper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Target Forward Testing Skripsi</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>100 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Awal Evaluasi</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>$500.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Terkini</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$498.68 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Total Trade Otomatis Selesai</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>7 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Progres Evaluasi (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>7.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade WIN (Profit)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>3 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade LOSS (Rugi)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>4 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Win Rate (%)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>42.86%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Total Akumulasi Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>$-1.32 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Return on Investment (ROI)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>-0.26%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Rata-rata Profit per Trade</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>$-0.19 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Waktu Pembaruan Terakhir</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-16 00:16:20 WIB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2578,12 +3816,840 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>2542162584</v>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 14:59:54</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 15:12:21</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>12m 27d</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>4310.915</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>4302.595</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>4323.195</v>
+      </c>
+      <c r="L31" s="3" t="n">
+        <v>4313.394</v>
+      </c>
+      <c r="M31" s="4" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>2542720557</v>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:24:54</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:31:27</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>1j 6m</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>4287.765</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>4277.635</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>4303.295</v>
+      </c>
+      <c r="L32" s="3" t="n">
+        <v>4289.619</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>2543321736</v>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:54:54</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 19:36:00</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>1j 41m</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>4291.905</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>4300.085</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>4279.885</v>
+      </c>
+      <c r="L33" s="3" t="n">
+        <v>4279.885</v>
+      </c>
+      <c r="M33" s="4" t="n">
+        <v>120.2</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>12.02</v>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P33" s="4" t="inlineStr">
+        <is>
+          <t>Hit Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="Q33" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2543302261</v>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 17:49:54</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 19:36:02</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>1j 46m</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>4292.741</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>4301.511</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>4279.651</v>
+      </c>
+      <c r="L34" s="3" t="n">
+        <v>4279.651</v>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>130.9</v>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>13.09</v>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P34" s="4" t="inlineStr">
+        <is>
+          <t>Hit Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>2544245058</v>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 19:59:53</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 20:08:14</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>8m 21d</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>4270.831</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>4257.741</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>4291.691</v>
+      </c>
+      <c r="L35" s="3" t="n">
+        <v>4257.741</v>
+      </c>
+      <c r="M35" s="4" t="n">
+        <v>-130.9</v>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>-13.09</v>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>2544403092</v>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 20:09:54</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 20:12:08</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>2m 14d</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>4260.791999999999</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>4246.312</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>4284.152</v>
+      </c>
+      <c r="L36" s="3" t="n">
+        <v>4263.284</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P36" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q36" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>2544587500</v>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 20:29:54</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 20:43:49</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>13m 55d</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>4272.991</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>4287.851</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>4248.941</v>
+      </c>
+      <c r="L37" s="3" t="n">
+        <v>4272.742999999999</v>
+      </c>
+      <c r="M37" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N37" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2544935748</v>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 21:04:53</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 21:14:51</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>9m 58d</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>4266.854</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>4281.076</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>4244.096</v>
+      </c>
+      <c r="L38" s="3" t="n">
+        <v>4281.076</v>
+      </c>
+      <c r="M38" s="4" t="n">
+        <v>-142.2</v>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>-14.23</v>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P38" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>2544686756</v>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 20:39:54</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 21:28:44</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>48m 50d</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>4268.914</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>4283.863</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>4244.563</v>
+      </c>
+      <c r="L39" s="3" t="n">
+        <v>4268.29</v>
+      </c>
+      <c r="M39" s="4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="N39" s="3" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>2545147164</v>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 21:24:53</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 21:48:48</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>23m 55d</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>4265.335</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>4279.515</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>4242.515</v>
+      </c>
+      <c r="L40" s="3" t="n">
+        <v>4279.515</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>-141.8</v>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>-14.18</v>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P40" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q40" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>2545450756</v>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 22:04:53</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 22:06:09</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>1m 16d</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>4273.633</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>4285.843</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>4254.353</v>
+      </c>
+      <c r="L41" s="3" t="n">
+        <v>4285.843</v>
+      </c>
+      <c r="M41" s="4" t="n">
+        <v>-122.1</v>
+      </c>
+      <c r="N41" s="3" t="n">
+        <v>-12.21</v>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P41" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>2546147073</v>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 23:29:55</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14 23:47:06</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>17m 11d</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>4300.285</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>4311.115</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>4283.495</v>
+      </c>
+      <c r="L42" s="3" t="n">
+        <v>4311.115</v>
+      </c>
+      <c r="M42" s="4" t="n">
+        <v>-108.3</v>
+      </c>
+      <c r="N42" s="3" t="n">
+        <v>-10.83</v>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="P42" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="Q42" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.5 (Macro + ATR)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2664,7 +4730,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>29 Trade</t>
+          <t>41 Trade</t>
         </is>
       </c>
     </row>
@@ -2676,7 +4742,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>41.0%</t>
         </is>
       </c>
     </row>
@@ -2688,7 +4754,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>16 Trade</t>
+          <t>23 Trade</t>
         </is>
       </c>
     </row>
@@ -2700,7 +4766,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>13 Trade</t>
+          <t>18 Trade</t>
         </is>
       </c>
     </row>
@@ -2712,7 +4778,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>55.17%</t>
+          <t>56.10%</t>
         </is>
       </c>
     </row>
@@ -2724,7 +4790,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>$+31.03 USD</t>
+          <t>$-0.72 USD</t>
         </is>
       </c>
     </row>
@@ -2736,7 +4802,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>$+1.07 USD</t>
+          <t>$-0.02 USD</t>
         </is>
       </c>
     </row>
@@ -2748,7 +4814,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>0.99</t>
         </is>
       </c>
     </row>
@@ -2760,7 +4826,931 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-14 13:55:38 WIB</t>
+          <t>2026-09-15 00:40:19 WIB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="53" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Trade Ke-</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Ticket Posisi</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Open</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Close</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Durasi</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Simbol</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Tipe</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Entry</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Exit</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Pips (P/L)</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>Saldo ($ USD)</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>Hasil</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t>Keterangan / Alasan Exit</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Model AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="n">
+        <v>2554812654</v>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 09:59:55</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 10:02:47</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>2m 52d</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I2" s="14" t="n">
+        <v>4320.834</v>
+      </c>
+      <c r="J2" s="14" t="n">
+        <v>4327.889</v>
+      </c>
+      <c r="K2" s="14" t="n">
+        <v>4308.289</v>
+      </c>
+      <c r="L2" s="14" t="n">
+        <v>4327.889</v>
+      </c>
+      <c r="M2" s="12" t="n">
+        <v>-70.59999999999999</v>
+      </c>
+      <c r="N2" s="14" t="n">
+        <v>-7.06</v>
+      </c>
+      <c r="O2" s="12" t="n">
+        <v>492.94</v>
+      </c>
+      <c r="P2" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q2" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R2" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="n">
+        <v>2557612722</v>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 19:54:55</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 20:12:45</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>17m 50d</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>4345.278</v>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>4352.027</v>
+      </c>
+      <c r="K3" s="14" t="n">
+        <v>4334.757</v>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>4352.027</v>
+      </c>
+      <c r="M3" s="12" t="n">
+        <v>-67.5</v>
+      </c>
+      <c r="N3" s="14" t="n">
+        <v>-6.75</v>
+      </c>
+      <c r="O3" s="12" t="n">
+        <v>486.19</v>
+      </c>
+      <c r="P3" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R3" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>2558074960</v>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 20:49:54</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 20:56:06</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>6m 12d</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>4342.834</v>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>4335.834</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>4355.434</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>4335.834</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N4" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O4" s="12" t="n">
+        <v>479.19</v>
+      </c>
+      <c r="P4" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R4" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>2560078028</v>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:19:54</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:22:19</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>2m 25d</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>4318.059999999999</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>4310.979</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>4330.579</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>4317.983</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="O5" s="12" t="n">
+        <v>479.11</v>
+      </c>
+      <c r="P5" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="R5" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>2564088044</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:49:53</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:12:32</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>22m 39d</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>4332.441</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>4339.441</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>4321.011</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>4321.011</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>11.43</v>
+      </c>
+      <c r="O6" s="9" t="n">
+        <v>490.54</v>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q6" s="10" t="inlineStr">
+        <is>
+          <t>Hit Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="R6" s="10" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>2564213179</v>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:14:53</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:32:11</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>17m 18d</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>4320.367999999999</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>4313.368</v>
+      </c>
+      <c r="K7" s="14" t="n">
+        <v>4332.178</v>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>4313.368</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N7" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O7" s="12" t="n">
+        <v>483.54</v>
+      </c>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R7" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>2565950780</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-17 19:59:54</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-17 20:00:32</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>0m 38d</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>4373.690000000001</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>4380.744</v>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>4361.144</v>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>4370.546</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="N8" s="11" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>486.68</v>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q8" s="10" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="R8" s="10" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>2566285253</v>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 20:34:53</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 20:38:06</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>3m 13d</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>4371.766</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>4364.766</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>4384.366</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>4364.766</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O9" s="12" t="n">
+        <v>479.68</v>
+      </c>
+      <c r="P9" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R9" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="84" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Metrik Evaluasi Forward Testing</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Nilai Evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Nama Model</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat) (28 Fitur SMC/ICT + DXY + MTF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Metode Eksekusi</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Otomatis 0-Delay (MetaTrader 5 API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ambang Batas Keyakinan (Threshold)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Versi 3.7 Multi-Zone Scalper (Wide SL + Sniper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Target Forward Testing Skripsi</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>100 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Awal Evaluasi</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>$500.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Terkini</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$479.68 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Total Trade Otomatis Selesai</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>8 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Progres Evaluasi (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>8.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade WIN (Profit)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>2 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade LOSS (Rugi)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>6 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Win Rate (%)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>25.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Total Akumulasi Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>$-20.32 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Return on Investment (ROI)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>-4.06%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Rata-rata Profit per Trade</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>$-2.54 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>0.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Waktu Pembaruan Terakhir</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-17 23:54:31 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(dashboard): isolasi progres skripsi hanya untuk model M15 dan pisahkan M5 sebagai non-skripsi
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -506,13 +506,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
@@ -526,7 +526,7 @@
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="53" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -618,6 +618,78 @@
       <c r="R1" s="7" t="inlineStr">
         <is>
           <t>Model AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="n">
+        <v>2573977759</v>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-19 00:14:54</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-19 00:34:25</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>19m 31d</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I2" s="14" t="n">
+        <v>4385.443</v>
+      </c>
+      <c r="J2" s="14" t="n">
+        <v>4392.443</v>
+      </c>
+      <c r="K2" s="14" t="n">
+        <v>4374.283</v>
+      </c>
+      <c r="L2" s="14" t="n">
+        <v>4392.443</v>
+      </c>
+      <c r="M2" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N2" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O2" s="12" t="n">
+        <v>493</v>
+      </c>
+      <c r="P2" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q2" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R2" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
         </is>
       </c>
     </row>
@@ -719,7 +791,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>$500.00 USD</t>
+          <t>$493.00 USD</t>
         </is>
       </c>
     </row>
@@ -731,7 +803,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>0 Trade</t>
+          <t>1 Trade</t>
         </is>
       </c>
     </row>
@@ -743,7 +815,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>1.0%</t>
         </is>
       </c>
     </row>
@@ -767,7 +839,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>0 Trade</t>
+          <t>1 Trade</t>
         </is>
       </c>
     </row>
@@ -791,7 +863,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>$+0.00 USD</t>
+          <t>$-7.00 USD</t>
         </is>
       </c>
     </row>
@@ -803,7 +875,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-1.40%</t>
         </is>
       </c>
     </row>
@@ -815,7 +887,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>$+0.00 USD</t>
+          <t>$-7.00 USD</t>
         </is>
       </c>
     </row>
@@ -827,7 +899,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.00</t>
         </is>
       </c>
     </row>
@@ -839,7 +911,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-19 00:14:55 WIB</t>
+          <t>2026-09-19 00:55:05 WIB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Figma Edition Modern Desktop & Web Dashboard, theme-adaptive icons, and portable setup
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -4,17 +4,19 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v3.7)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.7)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v3.6)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.6)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip v3.5)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.5)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip 16-17 Sep)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (Arsip 16-1" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v4.1)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v4.1)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v3.6)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.6)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip v3.5)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.5)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip 16-17 Sep)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (Arsip 16-1" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -526,7 +528,7 @@
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="53" customWidth="1" min="18" max="18"/>
+    <col width="49" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -689,7 +691,229 @@
       </c>
       <c r="R2" s="13" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+          <t>LightGBM M5 v4.0 (Trend-Aware + ADX + Volume)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="84" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Metrik Evaluasi Forward Testing</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Nilai Evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Nama Model</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat) (28 Fitur SMC/ICT + DXY + MTF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Metode Eksekusi</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Otomatis 0-Delay (MetaTrader 5 API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ambang Batas Keyakinan (Threshold)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Versi 3.7 Multi-Zone Scalper (Wide SL + Sniper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Target Forward Testing Skripsi</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>100 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Awal Evaluasi</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>$500.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Terkini</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$479.68 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Total Trade Otomatis Selesai</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>8 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Progres Evaluasi (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>8.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade WIN (Profit)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>2 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade LOSS (Rugi)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>6 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Win Rate (%)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>25.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Total Akumulasi Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>$-20.32 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Return on Investment (ROI)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>-4.06%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Rata-rata Profit per Trade</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>$-2.54 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>0.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Waktu Pembaruan Terakhir</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-17 23:54:31 WIB</t>
         </is>
       </c>
     </row>
@@ -708,7 +932,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="84" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -731,7 +955,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat) (28 Fitur SMC/ICT + DXY + MTF)</t>
+          <t>LightGBM M5 v4.0 (Trend-Aware + ADX + Volume) (28 Fitur SMC/ICT + DXY + MTF)</t>
         </is>
       </c>
     </row>
@@ -755,7 +979,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Versi 3.7 Multi-Zone Scalper (Wide SL + Sniper)</t>
+          <t>Versi 4.0 Multi-Zone Scalper (Trend-Aware)</t>
         </is>
       </c>
     </row>
@@ -911,7 +1135,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-19 00:55:05 WIB</t>
+          <t>2026-09-24 23:31:25 WIB</t>
         </is>
       </c>
     </row>
@@ -921,6 +1145,426 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="49" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Trade Ke-</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Ticket Posisi</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Open</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Close</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Durasi</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Simbol</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Tipe</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Entry</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Exit</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Pips (P/L)</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>Saldo ($ USD)</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>Hasil</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t>Keterangan / Alasan Exit</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Model AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="n">
+        <v>2573977759</v>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-19 00:14:54</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-19 00:34:25</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>19m 31d</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I2" s="14" t="n">
+        <v>4385.443</v>
+      </c>
+      <c r="J2" s="14" t="n">
+        <v>4392.443</v>
+      </c>
+      <c r="K2" s="14" t="n">
+        <v>4374.283</v>
+      </c>
+      <c r="L2" s="14" t="n">
+        <v>4392.443</v>
+      </c>
+      <c r="M2" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N2" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O2" s="12" t="n">
+        <v>493</v>
+      </c>
+      <c r="P2" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q2" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R2" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v4.0 (Trend-Aware + ADX + Volume)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Metrik Evaluasi Forward Testing</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Nilai Evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Nama Model</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v4.0 (Trend-Aware + ADX + Volume) (28 Fitur SMC/ICT + DXY + MTF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Metode Eksekusi</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Otomatis 0-Delay (MetaTrader 5 API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ambang Batas Keyakinan (Threshold)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Versi 4.0 Multi-Zone Scalper (Trend-Aware)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Target Forward Testing Skripsi</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>100 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Awal Evaluasi</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>$500.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Terkini</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$493.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Total Trade Otomatis Selesai</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>1 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Progres Evaluasi (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>1.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade WIN (Profit)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>0 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade LOSS (Rugi)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>1 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Win Rate (%)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Total Akumulasi Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>$-7.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Return on Investment (ROI)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>-1.40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Rata-rata Profit per Trade</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>$-7.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Waktu Pembaruan Terakhir</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-26 03:55:12 WIB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1550,7 +2194,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1772,7 +2416,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4721,7 +5365,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4907,7 +5551,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5607,226 +6251,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="84" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>Metrik Evaluasi Forward Testing</t>
-        </is>
-      </c>
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Nilai Evaluasi</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Nama Model</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat) (28 Fitur SMC/ICT + DXY + MTF)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Metode Eksekusi</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Otomatis 0-Delay (MetaTrader 5 API)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Ambang Batas Keyakinan (Threshold)</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Versi 3.7 Multi-Zone Scalper (Wide SL + Sniper)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Target Forward Testing Skripsi</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>100 Trade</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Saldo Awal Evaluasi</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>$500.00 USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Saldo Terkini</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>$479.68 USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Total Trade Otomatis Selesai</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>8 Trade</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Progres Evaluasi (%)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>8.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Jumlah Trade WIN (Profit)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>2 Trade</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Jumlah Trade LOSS (Rugi)</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>6 Trade</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Win Rate (%)</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>25.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Total Akumulasi Profit ($ USD)</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>$-20.32 USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Return on Investment (ROI)</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>-4.06%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Rata-rata Profit per Trade</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>$-2.54 USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Profit Factor</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>0.42</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Waktu Pembaruan Terakhir</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-17 23:54:31 WIB</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Web dashboard mobile responsiveness, PRO equity curve & evaluation autopsy, dynamic statistics summary, and project reorganization
</commit_message>
<xml_diff>
--- a/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
+++ b/Laporan_Forward_Testing_Model_M5_Scalping.xlsx
@@ -4,19 +4,20 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v3.7)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.7)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v4.1)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v4.1)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v3.6)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.6)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip v3.5)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.5)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip 16-17 Sep)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (Arsip 16-1" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik M5 (v4.1)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.7)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v4.1)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v4.1)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 Scalping (v3.6)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.6)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip v3.5)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (v3.5)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log M5 (Arsip 16-17 Sep)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Statistik (Arsip 16-1" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -706,6 +707,708 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="53" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Trade Ke-</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Ticket Posisi</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Open</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Waktu Close</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Durasi</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Simbol</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Tipe</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Entry</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Harga Exit</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Pips (P/L)</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>Saldo ($ USD)</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>Hasil</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t>Keterangan / Alasan Exit</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Model AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="n">
+        <v>2554812654</v>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 09:59:55</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 10:02:47</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>2m 52d</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I2" s="14" t="n">
+        <v>4320.834</v>
+      </c>
+      <c r="J2" s="14" t="n">
+        <v>4327.889</v>
+      </c>
+      <c r="K2" s="14" t="n">
+        <v>4308.289</v>
+      </c>
+      <c r="L2" s="14" t="n">
+        <v>4327.889</v>
+      </c>
+      <c r="M2" s="12" t="n">
+        <v>-70.59999999999999</v>
+      </c>
+      <c r="N2" s="14" t="n">
+        <v>-7.06</v>
+      </c>
+      <c r="O2" s="12" t="n">
+        <v>492.94</v>
+      </c>
+      <c r="P2" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q2" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R2" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="n">
+        <v>2557612722</v>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 19:54:55</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 20:12:45</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>17m 50d</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I3" s="14" t="n">
+        <v>4345.278</v>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>4352.027</v>
+      </c>
+      <c r="K3" s="14" t="n">
+        <v>4334.757</v>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>4352.027</v>
+      </c>
+      <c r="M3" s="12" t="n">
+        <v>-67.5</v>
+      </c>
+      <c r="N3" s="14" t="n">
+        <v>-6.75</v>
+      </c>
+      <c r="O3" s="12" t="n">
+        <v>486.19</v>
+      </c>
+      <c r="P3" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R3" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>2558074960</v>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 20:49:54</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-16 20:56:06</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>6m 12d</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>4342.834</v>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>4335.834</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>4355.434</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>4335.834</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N4" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O4" s="12" t="n">
+        <v>479.19</v>
+      </c>
+      <c r="P4" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R4" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>2560078028</v>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:19:54</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:22:19</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>2m 25d</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>4318.059999999999</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>4310.979</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>4330.579</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>4317.983</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="O5" s="12" t="n">
+        <v>479.11</v>
+      </c>
+      <c r="P5" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="R5" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>2564088044</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:49:53</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:12:32</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>22m 39d</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>4332.441</v>
+      </c>
+      <c r="J6" s="11" t="n">
+        <v>4339.441</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>4321.011</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>4321.011</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>11.43</v>
+      </c>
+      <c r="O6" s="9" t="n">
+        <v>490.54</v>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q6" s="10" t="inlineStr">
+        <is>
+          <t>Hit Take Profit (TP)</t>
+        </is>
+      </c>
+      <c r="R6" s="10" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>2564213179</v>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:14:53</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 15:32:11</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>17m 18d</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>4320.367999999999</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>4313.368</v>
+      </c>
+      <c r="K7" s="14" t="n">
+        <v>4332.178</v>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>4313.368</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N7" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O7" s="12" t="n">
+        <v>483.54</v>
+      </c>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R7" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>2565950780</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-17 19:59:54</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-17 20:00:32</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>0m 38d</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>4373.690000000001</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>4380.744</v>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>4361.144</v>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>4370.546</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="N8" s="11" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>486.68</v>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="Q8" s="10" t="inlineStr">
+        <is>
+          <t>Bot Trailing Profit Lock</t>
+        </is>
+      </c>
+      <c r="R8" s="10" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>2566285253</v>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 20:34:53</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-17 20:38:06</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>3m 13d</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>4371.766</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>4364.766</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>4384.366</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>4364.766</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>-70</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="O9" s="12" t="n">
+        <v>479.68</v>
+      </c>
+      <c r="P9" s="12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+      <c r="R9" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -923,6 +1626,252 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="84" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Metrik Evaluasi Forward Testing</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Nilai Evaluasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Nama Model</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Macro Scalp + Sniper) (28 Fitur SMC/ICT + DXY + MTF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Metode Eksekusi</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Otomatis 0-Delay (MetaTrader 5 API)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ambang Batas Keyakinan (Threshold)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Versi 4.1 Multi-Zone Scalper (Dynamic RRR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Target Forward Testing Skripsi</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>100 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Awal Evaluasi</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>$500.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Terkini</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>$493.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Total Trade Otomatis Selesai</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>1 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Progres Evaluasi (%)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>1.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade WIN (Murni)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>0 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade BEP (Netral)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>0 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Jumlah Trade LOSS (Rugi)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>1 Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Win Rate Murni (%) [Win/(Win+Loss)]</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Win Rate Total (%) [Win/Total]</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Total Akumulasi Profit ($ USD)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>$-7.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Return on Investment (ROI)</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>-1.40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Rata-rata Profit per Trade</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>$-7.00 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Waktu Pembaruan Terakhir</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-08 03:48:38 WIB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1144,13 +2093,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1169,8 +2118,10 @@
     <col width="18" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="49" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="53" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1256,10 +2207,20 @@
       </c>
       <c r="Q1" s="7" t="inlineStr">
         <is>
+          <t>Close 75m ($)</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Validasi Model 75M</t>
+        </is>
+      </c>
+      <c r="S1" s="7" t="inlineStr">
+        <is>
           <t>Keterangan / Alasan Exit</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="T1" s="7" t="inlineStr">
         <is>
           <t>Model AI</t>
         </is>
@@ -1326,14 +2287,22 @@
           <t>LOSS</t>
         </is>
       </c>
-      <c r="Q2" s="13" t="inlineStr">
+      <c r="Q2" s="13" t="n">
+        <v>4380.96</v>
+      </c>
+      <c r="R2" s="13" t="inlineStr">
+        <is>
+          <t>BERHASIL (SELARAS)</t>
+        </is>
+      </c>
+      <c r="S2" s="13" t="inlineStr">
         <is>
           <t>Hit Stop Loss (SL)</t>
         </is>
       </c>
-      <c r="R2" s="13" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v4.0 (Trend-Aware + ADX + Volume)</t>
+      <c r="T2" s="13" t="inlineStr">
+        <is>
+          <t>LightGBM M5 v3.7 (Wide SL + Macro Scalp + Sniper)</t>
         </is>
       </c>
     </row>
@@ -1342,7 +2311,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1555,7 +2524,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-26 03:55:12 WIB</t>
+          <t>2026-09-29 15:42:08 WIB</t>
         </is>
       </c>
     </row>
@@ -1564,7 +2533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2194,7 +3163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2416,7 +3385,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5365,7 +6334,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5549,706 +6518,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="53" customWidth="1" min="18" max="18"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Trade Ke-</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>Ticket Posisi</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Waktu Open</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>Waktu Close</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>Durasi</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>Simbol</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Tipe</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
-          <t>Lot</t>
-        </is>
-      </c>
-      <c r="I1" s="7" t="inlineStr">
-        <is>
-          <t>Harga Entry</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>Stop Loss (SL)</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>Take Profit (TP)</t>
-        </is>
-      </c>
-      <c r="L1" s="7" t="inlineStr">
-        <is>
-          <t>Harga Exit</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>Pips (P/L)</t>
-        </is>
-      </c>
-      <c r="N1" s="7" t="inlineStr">
-        <is>
-          <t>Profit ($ USD)</t>
-        </is>
-      </c>
-      <c r="O1" s="7" t="inlineStr">
-        <is>
-          <t>Saldo ($ USD)</t>
-        </is>
-      </c>
-      <c r="P1" s="7" t="inlineStr">
-        <is>
-          <t>Hasil</t>
-        </is>
-      </c>
-      <c r="Q1" s="7" t="inlineStr">
-        <is>
-          <t>Keterangan / Alasan Exit</t>
-        </is>
-      </c>
-      <c r="R1" s="7" t="inlineStr">
-        <is>
-          <t>Model AI</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="12" t="n">
-        <v>2554812654</v>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-16 09:59:55</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-16 10:02:47</t>
-        </is>
-      </c>
-      <c r="E2" s="12" t="inlineStr">
-        <is>
-          <t>2m 52d</t>
-        </is>
-      </c>
-      <c r="F2" s="12" t="inlineStr">
-        <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="G2" s="12" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I2" s="14" t="n">
-        <v>4320.834</v>
-      </c>
-      <c r="J2" s="14" t="n">
-        <v>4327.889</v>
-      </c>
-      <c r="K2" s="14" t="n">
-        <v>4308.289</v>
-      </c>
-      <c r="L2" s="14" t="n">
-        <v>4327.889</v>
-      </c>
-      <c r="M2" s="12" t="n">
-        <v>-70.59999999999999</v>
-      </c>
-      <c r="N2" s="14" t="n">
-        <v>-7.06</v>
-      </c>
-      <c r="O2" s="12" t="n">
-        <v>492.94</v>
-      </c>
-      <c r="P2" s="12" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="Q2" s="13" t="inlineStr">
-        <is>
-          <t>Hit Stop Loss (SL)</t>
-        </is>
-      </c>
-      <c r="R2" s="13" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="12" t="n">
-        <v>2557612722</v>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-16 19:54:55</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-16 20:12:45</t>
-        </is>
-      </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>17m 50d</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="inlineStr">
-        <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="H3" s="14" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I3" s="14" t="n">
-        <v>4345.278</v>
-      </c>
-      <c r="J3" s="14" t="n">
-        <v>4352.027</v>
-      </c>
-      <c r="K3" s="14" t="n">
-        <v>4334.757</v>
-      </c>
-      <c r="L3" s="14" t="n">
-        <v>4352.027</v>
-      </c>
-      <c r="M3" s="12" t="n">
-        <v>-67.5</v>
-      </c>
-      <c r="N3" s="14" t="n">
-        <v>-6.75</v>
-      </c>
-      <c r="O3" s="12" t="n">
-        <v>486.19</v>
-      </c>
-      <c r="P3" s="12" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="Q3" s="13" t="inlineStr">
-        <is>
-          <t>Hit Stop Loss (SL)</t>
-        </is>
-      </c>
-      <c r="R3" s="13" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="12" t="n">
-        <v>2558074960</v>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-16 20:49:54</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-16 20:56:06</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>6m 12d</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I4" s="14" t="n">
-        <v>4342.834</v>
-      </c>
-      <c r="J4" s="14" t="n">
-        <v>4335.834</v>
-      </c>
-      <c r="K4" s="14" t="n">
-        <v>4355.434</v>
-      </c>
-      <c r="L4" s="14" t="n">
-        <v>4335.834</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>-70</v>
-      </c>
-      <c r="N4" s="14" t="n">
-        <v>-7</v>
-      </c>
-      <c r="O4" s="12" t="n">
-        <v>479.19</v>
-      </c>
-      <c r="P4" s="12" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Hit Stop Loss (SL)</t>
-        </is>
-      </c>
-      <c r="R4" s="13" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>2560078028</v>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-17 01:19:54</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-17 01:22:19</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>2m 25d</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I5" s="14" t="n">
-        <v>4318.059999999999</v>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>4310.979</v>
-      </c>
-      <c r="K5" s="14" t="n">
-        <v>4330.579</v>
-      </c>
-      <c r="L5" s="14" t="n">
-        <v>4317.983</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-0.8</v>
-      </c>
-      <c r="N5" s="14" t="n">
-        <v>-0.08</v>
-      </c>
-      <c r="O5" s="12" t="n">
-        <v>479.11</v>
-      </c>
-      <c r="P5" s="12" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Bot Trailing Profit Lock</t>
-        </is>
-      </c>
-      <c r="R5" s="13" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="9" t="n">
-        <v>2564088044</v>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>2026-09-17 14:49:53</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:12:32</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>22m 39d</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I6" s="11" t="n">
-        <v>4332.441</v>
-      </c>
-      <c r="J6" s="11" t="n">
-        <v>4339.441</v>
-      </c>
-      <c r="K6" s="11" t="n">
-        <v>4321.011</v>
-      </c>
-      <c r="L6" s="11" t="n">
-        <v>4321.011</v>
-      </c>
-      <c r="M6" s="9" t="n">
-        <v>114.3</v>
-      </c>
-      <c r="N6" s="11" t="n">
-        <v>11.43</v>
-      </c>
-      <c r="O6" s="9" t="n">
-        <v>490.54</v>
-      </c>
-      <c r="P6" s="9" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="Q6" s="10" t="inlineStr">
-        <is>
-          <t>Hit Take Profit (TP)</t>
-        </is>
-      </c>
-      <c r="R6" s="10" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>2564213179</v>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:14:53</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-17 15:32:11</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>17m 18d</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I7" s="14" t="n">
-        <v>4320.367999999999</v>
-      </c>
-      <c r="J7" s="14" t="n">
-        <v>4313.368</v>
-      </c>
-      <c r="K7" s="14" t="n">
-        <v>4332.178</v>
-      </c>
-      <c r="L7" s="14" t="n">
-        <v>4313.368</v>
-      </c>
-      <c r="M7" s="12" t="n">
-        <v>-70</v>
-      </c>
-      <c r="N7" s="14" t="n">
-        <v>-7</v>
-      </c>
-      <c r="O7" s="12" t="n">
-        <v>483.54</v>
-      </c>
-      <c r="P7" s="12" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>Hit Stop Loss (SL)</t>
-        </is>
-      </c>
-      <c r="R7" s="13" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>2565950780</v>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>2026-09-17 19:59:54</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>2026-09-17 20:00:32</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>0m 38d</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I8" s="11" t="n">
-        <v>4373.690000000001</v>
-      </c>
-      <c r="J8" s="11" t="n">
-        <v>4380.744</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>4361.144</v>
-      </c>
-      <c r="L8" s="11" t="n">
-        <v>4370.546</v>
-      </c>
-      <c r="M8" s="9" t="n">
-        <v>31.4</v>
-      </c>
-      <c r="N8" s="11" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="O8" s="9" t="n">
-        <v>486.68</v>
-      </c>
-      <c r="P8" s="9" t="inlineStr">
-        <is>
-          <t>WIN</t>
-        </is>
-      </c>
-      <c r="Q8" s="10" t="inlineStr">
-        <is>
-          <t>Bot Trailing Profit Lock</t>
-        </is>
-      </c>
-      <c r="R8" s="10" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>2566285253</v>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-17 20:34:53</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>2026-09-17 20:38:06</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>3m 13d</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>XAUUSD</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>BUY</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I9" s="14" t="n">
-        <v>4371.766</v>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>4364.766</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>4384.366</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>4364.766</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>-70</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>-7</v>
-      </c>
-      <c r="O9" s="12" t="n">
-        <v>479.68</v>
-      </c>
-      <c r="P9" s="12" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>Hit Stop Loss (SL)</t>
-        </is>
-      </c>
-      <c r="R9" s="13" t="inlineStr">
-        <is>
-          <t>LightGBM M5 v3.7 (Wide SL + Sniper + Anti-Repeat)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>